<commit_message>
Mejoras en el prompt de corrección y en el de estructuración de la rúbrica
</commit_message>
<xml_diff>
--- a/docs/dataset-korrijo/prueba_1/rubrica.xlsx
+++ b/docs/dataset-korrijo/prueba_1/rubrica.xlsx
@@ -48,15 +48,15 @@
   </si>
   <si>
     <t xml:space="preserve">Bien
-(70%)</t>
+(75%)</t>
   </si>
   <si>
     <t xml:space="preserve">Básico
-(40%)</t>
+(45%)</t>
   </si>
   <si>
     <t xml:space="preserve">Insuficiente
-(10%)</t>
+(25%)</t>
   </si>
   <si>
     <t xml:space="preserve">No contesta /
@@ -76,16 +76,16 @@
     <t xml:space="preserve">Explica la vida nómada en el Paleolítico</t>
   </si>
   <si>
-    <t xml:space="preserve">Menciona las 3 actividades (caza, pesca, recolección), explica cómo condicionaban el desplazamiento del grupo y aporta al menos un detalle adicional (tamaño del grupo, tipo de refugio, etc.).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Menciona las 3 actividades y explica su relación con el nomadismo, sin detalles adicionales.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Menciona al menos 2 actividades y establece alguna relación con el desplazamiento del grupo.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Menciona actividades de subsistencia sin relacionarlas con el nomadismo, o la respuesta es muy incompleta.</t>
+    <t xml:space="preserve">Menciona las actividades de subsistencia (caza, pesca, recolección) y explica cómo se relacionaban con el desplazamiento del grupo nómada.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Menciona al menos dos actividades de subsistencia y las relaciona con el nomadismo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Menciona alguna actividad de subsistencia y la relaciona, aunque sea de forma general, con el desplazamiento del grupo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Menciona alguna actividad de subsistencia del Paleolítico, aunque no la conecte con el nomadismo.</t>
   </si>
   <si>
     <t xml:space="preserve">No contesta, la respuesta es incorrecta o totalmente irrelevante.</t>
@@ -97,16 +97,16 @@
     <t xml:space="preserve">Papel de la agricultura en el paso al sedentarismo</t>
   </si>
   <si>
-    <t xml:space="preserve">Explica qué es la agricultura, qué cambio supuso respecto a la recolección (producción propia) y por qué permitió establecerse en un lugar fijo.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Explica que la agricultura permitió producir alimento propio y relaciona esto con el sedentarismo, sin profundizar.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Menciona la agricultura como causa del sedentarismo pero sin explicar el mecanismo.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Menciona la agricultura de forma vaga, sin conexión clara con el sedentarismo.</t>
+    <t xml:space="preserve">Explica qué es la agricultura y por qué producir el propio alimento permitió a los grupos establecerse en un lugar fijo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Relaciona la agricultura con la producción de alimento propio y con el sedentarismo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Menciona la agricultura como causa del sedentarismo, aunque no explique bien el mecanismo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Menciona la agricultura en relación con la Prehistoria, aunque la conexión con el sedentarismo sea vaga.</t>
   </si>
   <si>
     <t xml:space="preserve">No contesta o la respuesta es incorrecta.</t>
@@ -115,16 +115,16 @@
     <t xml:space="preserve">Papel de la ganadería en el paso al sedentarismo</t>
   </si>
   <si>
-    <t xml:space="preserve">Explica qué aportó la ganadería (carne, leche, fuerza de trabajo, lana) y cómo complementó a la agricultura para fijar a los grupos humanos.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Menciona la ganadería como fuente de alimento controlado y la relaciona con el sedentarismo.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Menciona la domesticación de animales sin explicar cómo contribuyó al sedentarismo.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Menciona la ganadería de forma muy vaga o confusa.</t>
+    <t xml:space="preserve">Explica qué aportó la ganadería (alimento, fuerza de trabajo, lana...) y cómo ayudó a fijar a los grupos humanos.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Relaciona la ganadería con un aporte de alimento o recursos y con el sedentarismo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Menciona la domesticación de animales en relación con el modo de vida, aunque no explique su aporte al sedentarismo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Menciona la ganadería de forma general en el contexto de la Prehistoria.</t>
   </si>
   <si>
     <t xml:space="preserve">3</t>
@@ -133,16 +133,16 @@
     <t xml:space="preserve">Edad del Cobre: características y ventaja tecnológica</t>
   </si>
   <si>
-    <t xml:space="preserve">Nombra el período correctamente, explica que fue el primer metal trabajado, menciona su maleabilidad y señala su principal limitación (blandura, coexistencia con utensilios de piedra).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nombra el período, identifica el cobre como primer metal y señala una ventaja o limitación.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Menciona el cobre como metal de la primera etapa pero sin explicar ventaja ni limitación.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Menciona el cobre en el contexto de los metales pero de forma muy imprecisa.</t>
+    <t xml:space="preserve">Nombra el período e identifica el cobre como primer metal trabajado, señalando alguna característica (maleabilidad) o limitación.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nombra el período e identifica el cobre como primer metal trabajado.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Menciona el cobre como metal de la primera etapa de los metales.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Menciona el cobre dentro del contexto de la Prehistoria, aunque de forma imprecisa.</t>
   </si>
   <si>
     <t xml:space="preserve">No contesta, omite esta etapa o la respuesta es incorrecta.</t>
@@ -151,31 +151,31 @@
     <t xml:space="preserve">Edad del Bronce: características y ventaja tecnológica</t>
   </si>
   <si>
-    <t xml:space="preserve">Explica que el bronce es una aleación (cobre + estaño), indica que es más duro que el cobre, menciona la mejora en armas y herramientas y señala el impacto en el comercio (escasez de estaño).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Explica que el bronce es más duro que el cobre y que es una aleación, sin mencionar el comercio.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Menciona el bronce como mejora respecto al cobre pero sin explicar por qué (aleación) ni en qué consiste la mejora.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Menciona el bronce como etapa intermedia sin aportar ninguna explicación de su ventaja.</t>
+    <t xml:space="preserve">Explica que el bronce es una aleación más dura que el cobre y menciona su mejora en armas y herramientas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Indica que el bronce es más duro que el cobre y/o que es una aleación.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Menciona el bronce como una mejora respecto al cobre.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Menciona el bronce como una de las etapas de los metales.</t>
   </si>
   <si>
     <t xml:space="preserve">Edad del Hierro: características y ventaja tecnológica</t>
   </si>
   <si>
-    <t xml:space="preserve">Indica que el hierro es más abundante, más duro que el bronce, requería temperaturas más altas de fundición, y democratizó el acceso a herramientas y armas.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Indica que el hierro es más duro y más abundante que el bronce.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Menciona el hierro como el metal más avanzado sin explicar por qué supera al bronce.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Menciona el hierro como la última etapa de los metales sin ninguna explicación.</t>
+    <t xml:space="preserve">Indica que el hierro es más duro y más abundante que el bronce y que amplió el acceso a herramientas y armas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Indica que el hierro es más duro o más abundante que el bronce.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Menciona el hierro como el metal más avanzado de la etapa.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Menciona el hierro como una de las etapas de los metales.</t>
   </si>
   <si>
     <t xml:space="preserve">4</t>
@@ -184,16 +184,16 @@
     <t xml:space="preserve">Identificación del evento que marca el fin de la Prehistoria</t>
   </si>
   <si>
-    <t xml:space="preserve">Identifica correctamente la invención de la escritura (~3500 a.C., sumerios en Mesopotamia) como el hito que separa Prehistoria e Historia.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Identifica la escritura como el hito, sin precisar fecha ni lugar de origen.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Menciona algún evento relacionado (ciudades, civilizaciones) sin identificar la escritura explícitamente.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">La respuesta es vaga o confusa sobre cuál es el evento.</t>
+    <t xml:space="preserve">Identifica la invención de la escritura como el hito que separa Prehistoria e Historia (se valora, pero no se exige, precisar fecha o lugar).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Identifica la escritura como el hito que marca el fin de la Prehistoria.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Relaciona el fin de la Prehistoria con la escritura o con la aparición de las primeras civilizaciones o ciudades.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apunta algún evento relacionado con el cambio, aunque no identifique la escritura.</t>
   </si>
   <si>
     <t xml:space="preserve">No contesta o identifica un evento incorrecto.</t>
@@ -202,16 +202,16 @@
     <t xml:space="preserve">Análisis del impacto de la escritura</t>
   </si>
   <si>
-    <t xml:space="preserve">Explica al menos 3 impactos concretos de la escritura (registro de leyes/comercio, transmisión del conocimiento, administración de ciudades, surgimiento del escriba) y los conecta con el cambio social.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Explica 2 impactos concretos con cierto desarrollo.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Menciona 1 impacto concreto o enumera varios sin desarrollarlos.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Menciona que la escritura fue importante sin explicar en qué sentido.</t>
+    <t xml:space="preserve">Explica al menos dos impactos concretos de la escritura (registro de leyes o comercio, transmisión del conocimiento, administración...) conectándolos con el cambio social.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Explica uno o dos impactos concretos de la escritura.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Menciona algún impacto concreto de la escritura, aunque sin desarrollarlo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Menciona que la escritura fue importante, aunque no explique mucho en qué sentido.</t>
   </si>
   <si>
     <t xml:space="preserve">PUNTUACIÓN TOTAL</t>
@@ -223,25 +223,25 @@
     <t xml:space="preserve">Excelente (100%)</t>
   </si>
   <si>
-    <t xml:space="preserve">Respuesta completa, correcta y bien desarrollada. Demuestra comprensión profunda del concepto.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bien (70%)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Respuesta correcta en lo esencial, con alguna omisión menor o falta de desarrollo.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Básico (40%)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Respuesta parcialmente correcta. Identifica el concepto pero con errores o desarrollo insuficiente.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Insuficiente (10%)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Respuesta muy incompleta o con errores importantes. Solo demuestra un conocimiento muy superficial.</t>
+    <t xml:space="preserve">Respuesta correcta y bien planteada. Demuestra que se ha entendido el concepto, aunque no agote todos los detalles.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bien (75%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Respuesta correcta en lo esencial, aunque tenga omisiones o le falte algo de desarrollo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Básico (45%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Identifica el concepto y va encaminada, aunque el desarrollo sea breve o tenga alguna imprecisión.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Insuficiente (25%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Respuesta incompleta pero que apunta algo relacionado con el concepto.</t>
   </si>
   <si>
     <t xml:space="preserve">No contesta / Incorrecto (0%)</t>
@@ -254,9 +254,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="General"/>
   </numFmts>
   <fonts count="13">
     <font>
@@ -483,11 +482,15 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="33">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -560,11 +563,11 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="11" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -865,417 +868,415 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:J19"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.68359375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="32"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="4" style="0" width="38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="4" style="1" width="38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="30"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="3" t="s">
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="4" t="s">
+      <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
+      <c r="H2" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="4"/>
-      <c r="J2" s="4"/>
+      <c r="I2" s="5"/>
+      <c r="J2" s="5"/>
     </row>
     <row r="3" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="F3" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="G3" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="H3" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="I3" s="5" t="s">
+      <c r="I3" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="J3" s="5" t="s">
+      <c r="J3" s="6" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="6" t="n">
+      <c r="C4" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="D4" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="E4" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="F4" s="10" t="s">
+      <c r="F4" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="G4" s="11" t="s">
+      <c r="G4" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="H4" s="12" t="s">
+      <c r="H4" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="I4" s="13"/>
-      <c r="J4" s="14"/>
+      <c r="I4" s="14"/>
+      <c r="J4" s="15"/>
     </row>
     <row r="5" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="15" t="s">
+      <c r="A5" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="B5" s="16" t="s">
+      <c r="B5" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="C5" s="15" t="n">
+      <c r="C5" s="16" t="n">
         <v>1.25</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="D5" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="E5" s="9" t="s">
+      <c r="E5" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="F5" s="10" t="s">
+      <c r="F5" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="G5" s="11" t="s">
+      <c r="G5" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="H5" s="12" t="s">
+      <c r="H5" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="I5" s="13"/>
-      <c r="J5" s="17"/>
+      <c r="I5" s="14"/>
+      <c r="J5" s="18"/>
     </row>
     <row r="6" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="15" t="s">
+      <c r="A6" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="B6" s="16" t="s">
+      <c r="B6" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="C6" s="15" t="n">
+      <c r="C6" s="16" t="n">
         <v>1.25</v>
       </c>
-      <c r="D6" s="8" t="s">
+      <c r="D6" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="E6" s="9" t="s">
+      <c r="E6" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="F6" s="10" t="s">
+      <c r="F6" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="G6" s="11" t="s">
+      <c r="G6" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="H6" s="12" t="s">
+      <c r="H6" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="I6" s="13"/>
-      <c r="J6" s="17"/>
+      <c r="I6" s="14"/>
+      <c r="J6" s="18"/>
     </row>
     <row r="7" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="s">
+      <c r="A7" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="C7" s="6" t="n">
+      <c r="C7" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="D7" s="8" t="s">
+      <c r="D7" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="E7" s="9" t="s">
+      <c r="E7" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="F7" s="10" t="s">
+      <c r="F7" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="G7" s="11" t="s">
+      <c r="G7" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="H7" s="12" t="s">
+      <c r="H7" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="I7" s="13"/>
-      <c r="J7" s="14"/>
+      <c r="I7" s="14"/>
+      <c r="J7" s="15"/>
     </row>
     <row r="8" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="6" t="s">
+      <c r="A8" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="C8" s="6" t="n">
+      <c r="C8" s="7" t="n">
         <v>1.25</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="D8" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="E8" s="9" t="s">
+      <c r="E8" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="F8" s="10" t="s">
+      <c r="F8" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="G8" s="11" t="s">
+      <c r="G8" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="H8" s="12" t="s">
+      <c r="H8" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="I8" s="13"/>
-      <c r="J8" s="14"/>
+      <c r="I8" s="14"/>
+      <c r="J8" s="15"/>
     </row>
     <row r="9" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="s">
+      <c r="A9" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="C9" s="6" t="n">
+      <c r="C9" s="7" t="n">
         <v>1.25</v>
       </c>
-      <c r="D9" s="8" t="s">
+      <c r="D9" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="E9" s="9" t="s">
+      <c r="E9" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="F9" s="10" t="s">
+      <c r="F9" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="G9" s="11" t="s">
+      <c r="G9" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="H9" s="12" t="s">
+      <c r="H9" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="I9" s="13"/>
-      <c r="J9" s="14"/>
+      <c r="I9" s="14"/>
+      <c r="J9" s="15"/>
     </row>
     <row r="10" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="15" t="s">
+      <c r="A10" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="B10" s="16" t="s">
+      <c r="B10" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="C10" s="15" t="n">
+      <c r="C10" s="16" t="n">
         <v>0.5</v>
       </c>
-      <c r="D10" s="8" t="s">
+      <c r="D10" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="E10" s="9" t="s">
+      <c r="E10" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="F10" s="10" t="s">
+      <c r="F10" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="G10" s="11" t="s">
+      <c r="G10" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="H10" s="12" t="s">
+      <c r="H10" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="I10" s="13"/>
-      <c r="J10" s="17"/>
+      <c r="I10" s="14"/>
+      <c r="J10" s="18"/>
     </row>
     <row r="11" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="15" t="s">
+      <c r="A11" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="B11" s="16" t="s">
+      <c r="B11" s="17" t="s">
         <v>57</v>
       </c>
-      <c r="C11" s="15" t="n">
+      <c r="C11" s="16" t="n">
         <v>1.5</v>
       </c>
-      <c r="D11" s="8" t="s">
+      <c r="D11" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="E11" s="9" t="s">
+      <c r="E11" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="F11" s="10" t="s">
+      <c r="F11" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="G11" s="11" t="s">
+      <c r="G11" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="H11" s="12" t="s">
+      <c r="H11" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="I11" s="13"/>
-      <c r="J11" s="17"/>
+      <c r="I11" s="14"/>
+      <c r="J11" s="18"/>
     </row>
     <row r="12" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="18" t="s">
+      <c r="A12" s="19" t="s">
         <v>62</v>
       </c>
-      <c r="B12" s="18"/>
-      <c r="C12" s="19" t="n">
-        <f aca="false">SUM(C4:C11)</f>
+      <c r="B12" s="19"/>
+      <c r="C12" s="20" t="n">
         <v>10</v>
       </c>
-      <c r="D12" s="20"/>
-      <c r="E12" s="20"/>
-      <c r="F12" s="20"/>
-      <c r="G12" s="20"/>
-      <c r="H12" s="20"/>
-      <c r="I12" s="19" t="n">
-        <f aca="false">SUM(I4,I5,I6,I7,I8,I9,I10,I11)</f>
+      <c r="D12" s="21"/>
+      <c r="E12" s="21"/>
+      <c r="F12" s="21"/>
+      <c r="G12" s="21"/>
+      <c r="H12" s="21"/>
+      <c r="I12" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="J12" s="20"/>
+      <c r="J12" s="21"/>
     </row>
     <row r="14" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="21" t="s">
+      <c r="A14" s="22" t="s">
         <v>63</v>
       </c>
-      <c r="B14" s="21"/>
-      <c r="C14" s="21"/>
-      <c r="D14" s="21"/>
-      <c r="E14" s="21"/>
-      <c r="F14" s="21"/>
-      <c r="G14" s="21"/>
-      <c r="H14" s="21"/>
-      <c r="I14" s="21"/>
-      <c r="J14" s="21"/>
+      <c r="B14" s="22"/>
+      <c r="C14" s="22"/>
+      <c r="D14" s="22"/>
+      <c r="E14" s="22"/>
+      <c r="F14" s="22"/>
+      <c r="G14" s="22"/>
+      <c r="H14" s="22"/>
+      <c r="I14" s="22"/>
+      <c r="J14" s="22"/>
     </row>
     <row r="15" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="22" t="s">
+      <c r="A15" s="23" t="s">
         <v>64</v>
       </c>
-      <c r="B15" s="22"/>
-      <c r="C15" s="22"/>
-      <c r="D15" s="23" t="s">
+      <c r="B15" s="23"/>
+      <c r="C15" s="23"/>
+      <c r="D15" s="24" t="s">
         <v>65</v>
       </c>
-      <c r="E15" s="23"/>
-      <c r="F15" s="23"/>
-      <c r="G15" s="23"/>
-      <c r="H15" s="23"/>
-      <c r="I15" s="23"/>
-      <c r="J15" s="23"/>
+      <c r="E15" s="24"/>
+      <c r="F15" s="24"/>
+      <c r="G15" s="24"/>
+      <c r="H15" s="24"/>
+      <c r="I15" s="24"/>
+      <c r="J15" s="24"/>
     </row>
     <row r="16" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="24" t="s">
+      <c r="A16" s="25" t="s">
         <v>66</v>
       </c>
-      <c r="B16" s="24"/>
-      <c r="C16" s="24"/>
-      <c r="D16" s="25" t="s">
+      <c r="B16" s="25"/>
+      <c r="C16" s="25"/>
+      <c r="D16" s="26" t="s">
         <v>67</v>
       </c>
-      <c r="E16" s="25"/>
-      <c r="F16" s="25"/>
-      <c r="G16" s="25"/>
-      <c r="H16" s="25"/>
-      <c r="I16" s="25"/>
-      <c r="J16" s="25"/>
+      <c r="E16" s="26"/>
+      <c r="F16" s="26"/>
+      <c r="G16" s="26"/>
+      <c r="H16" s="26"/>
+      <c r="I16" s="26"/>
+      <c r="J16" s="26"/>
     </row>
     <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="26" t="s">
+      <c r="A17" s="27" t="s">
         <v>68</v>
       </c>
-      <c r="B17" s="26"/>
-      <c r="C17" s="26"/>
-      <c r="D17" s="27" t="s">
+      <c r="B17" s="27"/>
+      <c r="C17" s="27"/>
+      <c r="D17" s="28" t="s">
         <v>69</v>
       </c>
-      <c r="E17" s="27"/>
-      <c r="F17" s="27"/>
-      <c r="G17" s="27"/>
-      <c r="H17" s="27"/>
-      <c r="I17" s="27"/>
-      <c r="J17" s="27"/>
+      <c r="E17" s="28"/>
+      <c r="F17" s="28"/>
+      <c r="G17" s="28"/>
+      <c r="H17" s="28"/>
+      <c r="I17" s="28"/>
+      <c r="J17" s="28"/>
     </row>
     <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="28" t="s">
+      <c r="A18" s="29" t="s">
         <v>70</v>
       </c>
-      <c r="B18" s="28"/>
-      <c r="C18" s="28"/>
-      <c r="D18" s="29" t="s">
+      <c r="B18" s="29"/>
+      <c r="C18" s="29"/>
+      <c r="D18" s="30" t="s">
         <v>71</v>
       </c>
-      <c r="E18" s="29"/>
-      <c r="F18" s="29"/>
-      <c r="G18" s="29"/>
-      <c r="H18" s="29"/>
-      <c r="I18" s="29"/>
-      <c r="J18" s="29"/>
+      <c r="E18" s="30"/>
+      <c r="F18" s="30"/>
+      <c r="G18" s="30"/>
+      <c r="H18" s="30"/>
+      <c r="I18" s="30"/>
+      <c r="J18" s="30"/>
     </row>
     <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="30" t="s">
+      <c r="A19" s="31" t="s">
         <v>72</v>
       </c>
-      <c r="B19" s="30"/>
-      <c r="C19" s="30"/>
-      <c r="D19" s="31" t="s">
+      <c r="B19" s="31"/>
+      <c r="C19" s="31"/>
+      <c r="D19" s="32" t="s">
         <v>73</v>
       </c>
-      <c r="E19" s="31"/>
-      <c r="F19" s="31"/>
-      <c r="G19" s="31"/>
-      <c r="H19" s="31"/>
-      <c r="I19" s="31"/>
-      <c r="J19" s="31"/>
+      <c r="E19" s="32"/>
+      <c r="F19" s="32"/>
+      <c r="G19" s="32"/>
+      <c r="H19" s="32"/>
+      <c r="I19" s="32"/>
+      <c r="J19" s="32"/>
     </row>
   </sheetData>
   <mergeCells count="16">

</xml_diff>